<commit_message>
Finalize live fix validation and report evidence
</commit_message>
<xml_diff>
--- a/docs/BrainBox_Test_Execution_Report.xlsx
+++ b/docs/BrainBox_Test_Execution_Report.xlsx
@@ -1285,7 +1285,7 @@
       </c>
       <c r="H9" s="111" t="inlineStr">
         <is>
-          <t>Observed results captured on 2026-05-06 and follow-up fixes validated on 2026-05-07. Queue endpoint evidence corrected; web editor Home navigation fixed; web equation empty-line handling fixed; mobile playbar restore path fixed in code with live adb rerun still pending.</t>
+          <t>Observed results captured on 2026-05-06 and follow-up fixes validated on 2026-05-07. Queue endpoint evidence corrected; web editor Home navigation fixed and revalidated in a live browser rerun; web equation empty-line handling fixed and revalidated in a live browser rerun; mobile playbar restore path fixed and revalidated through a fresh adb/emulator rerun.</t>
         </is>
       </c>
     </row>
@@ -1447,7 +1447,7 @@
       </c>
       <c r="F3" s="111" t="inlineStr">
         <is>
-          <t>Known regression scenario remains in the plan.</t>
+          <t>Fixed (live rerun complete)</t>
         </is>
       </c>
       <c r="G3" s="111" t="inlineStr">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="H3" s="112" t="inlineStr">
         <is>
-          <t>Fixed on 2026-05-07 by replacing the full empty paragraph block before inserting block equations in the editor.</t>
+          <t>Authenticated browser rerun passed on 2026-05-07. Evidence: temp/fix-validation-2026-05-07/web-live-fix-evidence/summary.json plus equation-editing.png and equation-committed.png.</t>
         </is>
       </c>
       <c r="I3" s="112" t="inlineStr">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="F4" s="111" t="inlineStr">
         <is>
-          <t>Rerun the authenticated mobile shell, reach playlist/queue-adjacent surfaces, and attempt to restore active playback state.</t>
+          <t>Fixed (live rerun complete)</t>
         </is>
       </c>
       <c r="G4" s="111" t="inlineStr">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="H4" s="112" t="inlineStr">
         <is>
-          <t>Fixed on 2026-05-07 by restoring playback queue state during mobile home synchronization so the shell can render the global playbar when queue data exists.</t>
+          <t>Fresh Gradle tests passed and the adb/emulator rerun on 2026-05-07 showed the Playlist ready bar on Dashboard, Library, Quizzes, Flashcards, Playlist, and Profile after relaunch. Evidence: temp/fix-validation-2026-05-07/mobile-dashboard-playbar.png, mobile-library-playbar.xml, and mobile-playbar-tabs.json.</t>
         </is>
       </c>
       <c r="I4" s="112" t="inlineStr">
@@ -1551,7 +1551,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Open a notebook, make an unsaved change, and click the editor Home button.</t>
+          <t>Fixed (live rerun complete)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="H5" s="112" t="inlineStr">
         <is>
-          <t>Fixed on 2026-05-07 by saving pending edits and explicitly returning the user to /dashboard after save succeeds.</t>
+          <t>Authenticated browser rerun passed on 2026-05-07. Evidence: temp/fix-validation-2026-05-07/web-live-fix-evidence/summary.json and home-nav-dashboard.png.</t>
         </is>
       </c>
       <c r="I5" s="112" t="inlineStr">
@@ -2432,7 +2432,7 @@
     <row r="40">
       <c r="A40" s="111" t="inlineStr">
         <is>
-          <t>Open regressions remain limited to the queue HTTP 500 failure, the unsaved editor Home navigation defect, and the equation-tool known-risk scenario that still needs a targeted editor fixture.</t>
+          <t>Confirmed defects from the 06-07 May remediation set are now closed: the queue-endpoint evidence was corrected, the unsaved editor Home navigation defect was fixed, the empty-line equation regression was fixed, and the mobile playbar restore path passed a fresh live emulator rerun.</t>
         </is>
       </c>
       <c r="B40" s="111" t="inlineStr">
@@ -2442,7 +2442,7 @@
       </c>
       <c r="C40" s="111" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
     </row>
@@ -4454,7 +4454,7 @@
       </c>
       <c r="B3" s="112" t="inlineStr">
         <is>
-          <t>Document the remediation pass completed after the 2026-05-06 observed regression rerun. This sheet records which bugs were fixed, how they were revalidated, and which live reruns are still recommended.</t>
+          <t>Document the remediation pass completed after the 2026-05-06 observed regression rerun. This sheet records which bugs were fixed, how they were revalidated, and how the follow-up live reruns closed the remaining professor-facing evidence gaps.</t>
         </is>
       </c>
       <c r="C3" s="112" t="inlineStr"/>
@@ -4540,12 +4540,12 @@
       </c>
       <c r="D7" s="112" t="inlineStr">
         <is>
-          <t>temp/fix-validation-2026-05-07/web-node-test.log; temp/fix-validation-2026-05-07/web-vite-build.log</t>
+          <t>temp/fix-validation-2026-05-07/web-node-test.log; temp/fix-validation-2026-05-07/web-vite-build.log; temp/fix-validation-2026-05-07/web-live-fix-evidence/summary.json</t>
         </is>
       </c>
       <c r="E7" s="112" t="inlineStr">
         <is>
-          <t>Implemented on branch fix/web-editor-home-navigation.</t>
+          <t>Implemented on branch fix/web-editor-home-navigation and cleared by the authenticated browser rerun on 2026-05-07.</t>
         </is>
       </c>
     </row>
@@ -4567,12 +4567,12 @@
       </c>
       <c r="D8" s="112" t="inlineStr">
         <is>
-          <t>temp/fix-validation-2026-05-07/web-node-test.log; temp/fix-validation-2026-05-07/web-vite-build.log</t>
+          <t>temp/fix-validation-2026-05-07/web-node-test.log; temp/fix-validation-2026-05-07/web-vite-build.log; temp/fix-validation-2026-05-07/web-live-fix-evidence/summary.json</t>
         </is>
       </c>
       <c r="E8" s="112" t="inlineStr">
         <is>
-          <t>Implemented on branch fix/web-equation-empty-line. A targeted browser rerun is still recommended for live professor-facing evidence.</t>
+          <t>Implemented on branch fix/web-equation-empty-line and cleared by the authenticated browser rerun on 2026-05-07.</t>
         </is>
       </c>
     </row>
@@ -4584,7 +4584,7 @@
       </c>
       <c r="B9" s="112" t="inlineStr">
         <is>
-          <t>Fixed pending live rerun</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="C9" s="112" t="inlineStr">
@@ -4594,12 +4594,12 @@
       </c>
       <c r="D9" s="112" t="inlineStr">
         <is>
-          <t>temp/fix-validation-2026-05-07/mobile-gradle-test.log</t>
+          <t>temp/fix-validation-2026-05-07/mobile-gradle-test.log; temp/fix-validation-2026-05-07/mobile-dashboard-playbar.png; temp/fix-validation-2026-05-07/mobile-library-playbar.xml; temp/fix-validation-2026-05-07/mobile-playbar-tabs.json</t>
         </is>
       </c>
       <c r="E9" s="112" t="inlineStr">
         <is>
-          <t>Implemented on branch fix/mobile-playbar-visibility. adb was not available in the current environment, so no replacement emulator screenshot set was captured on 2026-05-07.</t>
+          <t>Implemented on branch fix/mobile-playbar-visibility and cleared by the adb/emulator rerun on 2026-05-07.</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="E16" s="112" t="inlineStr">
         <is>
-          <t>The available unit-related tasks passed; no fresh connected rerun was captured because adb was unavailable.</t>
+          <t>The available unit-related tasks passed, and the live adb/emulator UI rerun is documented separately below.</t>
         </is>
       </c>
     </row>
@@ -4814,22 +4814,22 @@
       </c>
       <c r="B19" s="112" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="C19" s="112" t="inlineStr">
         <is>
-          <t>Repeat the authenticated emulator playback scenario once adb or a device is available.</t>
+          <t>Authenticated emulator rerun showed the collapsed Playlist ready bar above bottom navigation after relaunch, including Dashboard and Library screenshot/XML capture plus tab persistence across Quizzes, Flashcards, Playlist, and Profile.</t>
         </is>
       </c>
       <c r="D19" s="112" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>temp/fix-validation-2026-05-07/mobile-dashboard-playbar.png; temp/fix-validation-2026-05-07/mobile-library-playbar.png; temp/fix-validation-2026-05-07/mobile-library-playbar.xml; temp/fix-validation-2026-05-07/mobile-playbar-tabs.json</t>
         </is>
       </c>
       <c r="E19" s="112" t="inlineStr">
         <is>
-          <t>Code fix is already in place; this gap is about replacing the older failed screenshot evidence.</t>
+          <t>The older failed mobile screenshot evidence has been replaced by a fresh live rerun set.</t>
         </is>
       </c>
     </row>
@@ -4841,22 +4841,22 @@
       </c>
       <c r="B20" s="112" t="inlineStr">
         <is>
-          <t>Recommended</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="C20" s="112" t="inlineStr">
         <is>
-          <t>Run an authenticated browser script that explicitly covers the Home button handoff and empty-line equation insertion.</t>
+          <t>Authenticated browser rerun covered the Home-button save handoff and empty-line block-equation path successfully.</t>
         </is>
       </c>
       <c r="D20" s="112" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>temp/fix-validation-2026-05-07/web-live-fix-evidence/summary.json; temp/fix-validation-2026-05-07/web-live-fix-evidence/home-nav-dashboard.png; temp/fix-validation-2026-05-07/web-live-fix-evidence/equation-editing.png; temp/fix-validation-2026-05-07/web-live-fix-evidence/equation-committed.png</t>
         </is>
       </c>
       <c r="E20" s="112" t="inlineStr">
         <is>
-          <t>Local web automation and production build already passed after the code fixes.</t>
+          <t>The targeted professor-facing browser rerun is complete.</t>
         </is>
       </c>
     </row>
@@ -15750,12 +15750,12 @@
       </c>
       <c r="I49" s="111" t="inlineStr">
         <is>
-          <t>Known regression risk remains open. The exact block-equation-on-empty-line scenario still requires a targeted fixture, so this case is marked Failed for the current execution run.</t>
+          <t>Authenticated browser rerun on 2026-05-07 passed. A blank paragraph accepted block equation insertion, the MathLive field stayed visible while typing, and the block equation committed successfully. Evidence: temp/fix-validation-2026-05-07/web-live-fix-evidence/summary.json plus equation-editing.png and equation-committed.png.</t>
         </is>
       </c>
       <c r="J49" s="98" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="K49" s="111" t="inlineStr">
@@ -16990,12 +16990,12 @@
       </c>
       <c r="I69" s="111" t="inlineStr">
         <is>
-          <t>Dashboard, playlist, and queue-adjacent surfaces reran on emulator-5554, but an active media session was not re-established after relaunch. The collapsed global playbar regression therefore remains Failed in this run.</t>
+          <t>Fresh adb/emulator rerun on 2026-05-07 passed. After queue restoration and relaunch, the collapsed Playlist ready bar was visible above bottom navigation on Dashboard, Library, Quizzes, Flashcards, Playlist, and Profile. Evidence: temp/fix-validation-2026-05-07/mobile-dashboard-playbar.png, mobile-library-playbar.xml, and mobile-playbar-tabs.json.</t>
         </is>
       </c>
       <c r="J69" s="98" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="K69" s="111" t="inlineStr">
@@ -18230,12 +18230,12 @@
       </c>
       <c r="I89" s="111" t="inlineStr">
         <is>
-          <t>Known regression recorded for the current build: clicking Home from an unsaved notebook triggers a save but does not route the user back to the home surface. No fix was applied in this pass.</t>
+          <t>Authenticated browser rerun on 2026-05-07 passed. Clicking Home from an unsaved notebook saved the edit and returned the user to /dashboard, and the notebook content remained persisted through the API. Evidence: temp/fix-validation-2026-05-07/web-live-fix-evidence/summary.json and home-nav-dashboard.png.</t>
         </is>
       </c>
       <c r="J89" s="95" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
     </row>
@@ -22805,12 +22805,12 @@
       </c>
       <c r="H101" s="98" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I101" s="111" t="inlineStr">
         <is>
-          <t>2026-05-06: Credential-based rerun - Known regression risk remains in the plan. The exact editor/mobile scenario requires a targeted fixture or attached device. No fix was attempted.</t>
+          <t>2026-05-07: Authenticated browser rerun passed. The empty-line block-equation path stayed stable from field creation through KaTeX commit. Evidence: temp/fix-validation-2026-05-07/web-live-fix-evidence/summary.json.</t>
         </is>
       </c>
     </row>
@@ -22850,12 +22850,12 @@
       </c>
       <c r="H102" s="98" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I102" s="111" t="inlineStr">
         <is>
-          <t>2026-05-06: Credential-based rerun - Known regression risk remains in the plan. The exact editor/mobile scenario requires a targeted fixture or attached device. No fix was attempted.</t>
+          <t>2026-05-07: Authenticated browser rerun passed. The empty-line block-equation path stayed stable from field creation through KaTeX commit. Evidence: temp/fix-validation-2026-05-07/web-live-fix-evidence/summary.json.</t>
         </is>
       </c>
     </row>
@@ -22895,12 +22895,12 @@
       </c>
       <c r="H103" s="98" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I103" s="111" t="inlineStr">
         <is>
-          <t>2026-05-06: Credential-based rerun - Known regression risk remains in the plan. The exact editor/mobile scenario requires a targeted fixture or attached device. No fix was attempted.</t>
+          <t>2026-05-07: Authenticated browser rerun passed. The empty-line block-equation path stayed stable from field creation through KaTeX commit. Evidence: temp/fix-validation-2026-05-07/web-live-fix-evidence/summary.json.</t>
         </is>
       </c>
     </row>
@@ -22925,7 +22925,7 @@
       </c>
       <c r="E104" s="111" t="inlineStr">
         <is>
-          <t>Press Enter or blur the equation field.</t>
+          <t>Press Shift+Enter or blur the equation field.</t>
         </is>
       </c>
       <c r="F104" s="111" t="inlineStr">
@@ -22940,12 +22940,12 @@
       </c>
       <c r="H104" s="98" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I104" s="111" t="inlineStr">
         <is>
-          <t>2026-05-06: Credential-based rerun - Known regression risk remains in the plan. The exact editor/mobile scenario requires a targeted fixture or attached device. No fix was attempted.</t>
+          <t>2026-05-07: Authenticated browser rerun passed. The empty-line block-equation path stayed stable from field creation through KaTeX commit. Evidence: temp/fix-validation-2026-05-07/web-live-fix-evidence/summary.json.</t>
         </is>
       </c>
     </row>
@@ -23390,12 +23390,12 @@
       </c>
       <c r="H114" s="98" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I114" s="111" t="inlineStr">
         <is>
-          <t>2026-05-06: Credential-based rerun - Known regression risk remains in the plan. The exact editor/mobile scenario requires a targeted fixture or attached device. No fix was attempted.</t>
+          <t>2026-05-07: Fresh adb/emulator rerun passed. The collapsed Playlist ready bar remained visible after relaunch and across Dashboard, Library, Quizzes, Flashcards, Playlist, and Profile. Evidence: temp/fix-validation-2026-05-07/mobile-dashboard-playbar.png, mobile-library-playbar.xml, and mobile-playbar-tabs.json.</t>
         </is>
       </c>
     </row>
@@ -23435,12 +23435,12 @@
       </c>
       <c r="H115" s="98" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I115" s="111" t="inlineStr">
         <is>
-          <t>2026-05-06: Credential-based rerun - Known regression risk remains in the plan. The exact editor/mobile scenario requires a targeted fixture or attached device. No fix was attempted.</t>
+          <t>2026-05-07: Fresh adb/emulator rerun passed. The collapsed Playlist ready bar remained visible after relaunch and across Dashboard, Library, Quizzes, Flashcards, Playlist, and Profile. Evidence: temp/fix-validation-2026-05-07/mobile-dashboard-playbar.png, mobile-library-playbar.xml, and mobile-playbar-tabs.json.</t>
         </is>
       </c>
     </row>
@@ -23480,12 +23480,12 @@
       </c>
       <c r="H116" s="98" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I116" s="111" t="inlineStr">
         <is>
-          <t>2026-05-06: Credential-based rerun - Known regression risk remains in the plan. The exact editor/mobile scenario requires a targeted fixture or attached device. No fix was attempted.</t>
+          <t>2026-05-07: Fresh adb/emulator rerun passed. The collapsed Playlist ready bar remained visible after relaunch and across Dashboard, Library, Quizzes, Flashcards, Playlist, and Profile. Evidence: temp/fix-validation-2026-05-07/mobile-dashboard-playbar.png, mobile-library-playbar.xml, and mobile-playbar-tabs.json.</t>
         </is>
       </c>
     </row>
@@ -31760,12 +31760,12 @@
       </c>
       <c r="H300" s="95" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I300" s="111" t="inlineStr">
         <is>
-          <t>2026-05-06: Known regression recorded for the current build. Clicking Home from an unsaved notebook saves the content but does not navigate back to the home surface. No fix was applied in this pass.</t>
+          <t>2026-05-07: Authenticated browser rerun passed. Clicking Home from an unsaved notebook saved the pending edit, returned the route to /dashboard, and preserved the new content through the notebook API. Evidence: temp/fix-validation-2026-05-07/web-live-fix-evidence/summary.json.</t>
         </is>
       </c>
     </row>
@@ -31805,12 +31805,12 @@
       </c>
       <c r="H301" s="95" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I301" s="111" t="inlineStr">
         <is>
-          <t>2026-05-06: Known regression recorded for the current build. Clicking Home from an unsaved notebook saves the content but does not navigate back to the home surface. No fix was applied in this pass.</t>
+          <t>2026-05-07: Authenticated browser rerun passed. Clicking Home from an unsaved notebook saved the pending edit, returned the route to /dashboard, and preserved the new content through the notebook API. Evidence: temp/fix-validation-2026-05-07/web-live-fix-evidence/summary.json.</t>
         </is>
       </c>
     </row>
@@ -31850,12 +31850,12 @@
       </c>
       <c r="H302" s="95" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I302" s="111" t="inlineStr">
         <is>
-          <t>2026-05-06: Known regression recorded for the current build. Clicking Home from an unsaved notebook saves the content but does not navigate back to the home surface. No fix was applied in this pass.</t>
+          <t>2026-05-07: Authenticated browser rerun passed. Clicking Home from an unsaved notebook saved the pending edit, returned the route to /dashboard, and preserved the new content through the notebook API. Evidence: temp/fix-validation-2026-05-07/web-live-fix-evidence/summary.json.</t>
         </is>
       </c>
     </row>
@@ -31895,12 +31895,12 @@
       </c>
       <c r="H303" s="95" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I303" s="111" t="inlineStr">
         <is>
-          <t>2026-05-06: Known regression recorded for the current build. Clicking Home from an unsaved notebook saves the content but does not navigate back to the home surface. No fix was applied in this pass.</t>
+          <t>2026-05-07: Authenticated browser rerun passed. Clicking Home from an unsaved notebook saved the pending edit, returned the route to /dashboard, and preserved the new content through the notebook API. Evidence: temp/fix-validation-2026-05-07/web-live-fix-evidence/summary.json.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update regression retest evidence
</commit_message>
<xml_diff>
--- a/docs/BrainBox_Test_Execution_Report.xlsx
+++ b/docs/BrainBox_Test_Execution_Report.xlsx
@@ -4402,7 +4402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4589,17 +4589,17 @@
       </c>
       <c r="C9" s="112" t="inlineStr">
         <is>
-          <t>Mobile home synchronization now restores playback queue state into the shell view state so the global playbar can render whenever an active queue exists.</t>
+          <t>Mobile home synchronization now restores playback queue state into the shell view state so the global playbar can render whenever an active queue exists, and the fallback copy now reads Playback ready during idle relaunch state.</t>
         </is>
       </c>
       <c r="D9" s="112" t="inlineStr">
         <is>
-          <t>temp/fix-validation-2026-05-07/mobile-gradle-test.log; temp/fix-validation-2026-05-07/mobile-dashboard-playbar.png; temp/fix-validation-2026-05-07/mobile-library-playbar.xml; temp/fix-validation-2026-05-07/mobile-playbar-tabs.json</t>
+          <t>temp/fix-validation-2026-05-07/mobile-gradle-test.log; temp/fix-validation-2026-05-07/dashboard-playback-ready-label-valid.png; temp/fix-validation-2026-05-07/dashboard-playback-ready-label-valid.xml; temp/fix-validation-2026-05-07/library-playbar-valid.png; temp/fix-validation-2026-05-07/library-playbar-rerun.xml; temp/fix-validation-2026-05-07/mobile-playbar-pause-rerun.json; temp/fix-validation-2026-05-07/mobile-playbar-resume-rerun.json</t>
         </is>
       </c>
       <c r="E9" s="112" t="inlineStr">
         <is>
-          <t>Implemented on branch fix/mobile-playbar-visibility and cleared by the adb/emulator rerun on 2026-05-07.</t>
+          <t>Implemented on branches fix/mobile-playbar-visibility and fix/mobile-playbar-label, then revalidated through the adb/emulator rerun on 07 May 2026.</t>
         </is>
       </c>
     </row>
@@ -4782,27 +4782,27 @@
     <row r="18">
       <c r="A18" s="116" t="inlineStr">
         <is>
-          <t>Remaining Validation Gaps</t>
+          <t>Mobile playbar live UI proof</t>
         </is>
       </c>
       <c r="B18" s="116" t="inlineStr">
         <is>
-          <t>Current State</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="C18" s="116" t="inlineStr">
         <is>
-          <t>Recommended Next Step</t>
+          <t>The 07 May rerun now includes a relaunch screenshot showing the updated Playback ready fallback state, plus fresh Dashboard and Library evidence proving the global playbar remains visible after navigation.</t>
         </is>
       </c>
       <c r="D18" s="116" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>temp/fix-validation-2026-05-07/dashboard-playback-ready-label-valid.png; temp/fix-validation-2026-05-07/dashboard-playback-ready-label-valid.xml; temp/fix-validation-2026-05-07/library-playbar-valid.png; temp/fix-validation-2026-05-07/library-playbar-rerun.xml</t>
         </is>
       </c>
       <c r="E18" s="116" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>The older Playlist ready wording is no longer present in the validated rerun evidence.</t>
         </is>
       </c>
     </row>
@@ -4857,6 +4857,222 @@
       <c r="E20" s="112" t="inlineStr">
         <is>
           <t>The targeted professor-facing browser rerun is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="116" t="inlineStr">
+        <is>
+          <t>Focused Live Retest 2026-05-07</t>
+        </is>
+      </c>
+      <c r="B22" s="116" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C22" s="116" t="inlineStr">
+        <is>
+          <t>Observed Result</t>
+        </is>
+      </c>
+      <c r="D22" s="116" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="E22" s="116" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="45" customHeight="1">
+      <c r="A23" s="112" t="inlineStr">
+        <is>
+          <t>Web editor Home navigation</t>
+        </is>
+      </c>
+      <c r="B23" s="112" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="C23" s="112" t="inlineStr">
+        <is>
+          <t>The editor Home control returned to /dashboard after saving the pending note change.</t>
+        </is>
+      </c>
+      <c r="D23" s="112" t="inlineStr">
+        <is>
+          <t>temp/fix-validation-2026-05-07/web-live-fix-evidence/home-nav-dashboard.png; temp/fix-validation-2026-05-07/web-live-fix-evidence/summary.json</t>
+        </is>
+      </c>
+      <c r="E23" s="112" t="inlineStr">
+        <is>
+          <t>Authenticated browser rerun with API-backed persistence assertion completed on 07 May 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="45" customHeight="1">
+      <c r="A24" s="112" t="inlineStr">
+        <is>
+          <t>Web empty-line equation insertion</t>
+        </is>
+      </c>
+      <c r="B24" s="112" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="C24" s="112" t="inlineStr">
+        <is>
+          <t>The display equation editor stayed visible while typing x^2+1 on a new empty line and rendered correctly after commit.</t>
+        </is>
+      </c>
+      <c r="D24" s="112" t="inlineStr">
+        <is>
+          <t>temp/fix-validation-2026-05-07/web-live-fix-evidence/equation-editing.png; temp/fix-validation-2026-05-07/web-live-fix-evidence/equation-committed.png; temp/fix-validation-2026-05-07/web-live-fix-evidence/summary.json</t>
+        </is>
+      </c>
+      <c r="E24" s="112" t="inlineStr">
+        <is>
+          <t>This is the fresh post-fix browser rerun requested for the appendix update.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="45" customHeight="1">
+      <c r="A25" s="112" t="inlineStr">
+        <is>
+          <t>Mobile fallback label copy</t>
+        </is>
+      </c>
+      <c r="B25" s="112" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="C25" s="112" t="inlineStr">
+        <is>
+          <t>A clean relaunch showed the idle playbar label as Playback ready with the Start playlist action.</t>
+        </is>
+      </c>
+      <c r="D25" s="112" t="inlineStr">
+        <is>
+          <t>temp/fix-validation-2026-05-07/dashboard-playback-ready-label-valid.png; temp/fix-validation-2026-05-07/dashboard-playback-ready-label-valid.xml</t>
+        </is>
+      </c>
+      <c r="E25" s="112" t="inlineStr">
+        <is>
+          <t>Confirms the follow-up UI copy change on fix/mobile-playbar-label.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="45" customHeight="1">
+      <c r="A26" s="112" t="inlineStr">
+        <is>
+          <t>Mobile playbar visibility across tabs</t>
+        </is>
+      </c>
+      <c r="B26" s="112" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="C26" s="112" t="inlineStr">
+        <is>
+          <t>The Library tab retained the global playbar with the seeded notebook title visible above bottom navigation.</t>
+        </is>
+      </c>
+      <c r="D26" s="112" t="inlineStr">
+        <is>
+          <t>temp/fix-validation-2026-05-07/library-playbar-valid.png; temp/fix-validation-2026-05-07/library-playbar-rerun.xml</t>
+        </is>
+      </c>
+      <c r="E26" s="112" t="inlineStr">
+        <is>
+          <t>Complements the dashboard capture and confirms the original visibility regression remains fixed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="45" customHeight="1">
+      <c r="A27" s="112" t="inlineStr">
+        <is>
+          <t>Mobile playbar pause and resume responsiveness</t>
+        </is>
+      </c>
+      <c r="B27" s="112" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="C27" s="112" t="inlineStr">
+        <is>
+          <t>Pause reached PAUSED in 67 ms and resume returned to PLAYING in 764 ms during the live emulator rerun.</t>
+        </is>
+      </c>
+      <c r="D27" s="112" t="inlineStr">
+        <is>
+          <t>temp/fix-validation-2026-05-07/mobile-playbar-paused-valid.png; temp/fix-validation-2026-05-07/mobile-playbar-resumed-valid.png; temp/fix-validation-2026-05-07/mobile-playbar-pause-rerun.json; temp/fix-validation-2026-05-07/mobile-playbar-resume-rerun.json</t>
+        </is>
+      </c>
+      <c r="E27" s="112" t="inlineStr">
+        <is>
+          <t>No user-visible lag was observed while interacting with the collapsed playbar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="45" customHeight="1">
+      <c r="A28" s="112" t="inlineStr">
+        <is>
+          <t>Mobile review-mode audio playback</t>
+        </is>
+      </c>
+      <c r="B28" s="112" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="C28" s="112" t="inlineStr">
+        <is>
+          <t>Review mode advanced from 0:00 to 0:07 of 0:37 while Android TTS and media-session logs were emitted.</t>
+        </is>
+      </c>
+      <c r="D28" s="112" t="inlineStr">
+        <is>
+          <t>temp/fix-validation-2026-05-07/review-audio-valid.png; temp/fix-validation-2026-05-07/review-audio-valid.xml; temp/fix-validation-2026-05-07/review-audio-valid.log</t>
+        </is>
+      </c>
+      <c r="E28" s="112" t="inlineStr">
+        <is>
+          <t>Confirms that the review-mode audio path is live on the emulator, not just statically rendered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="45" customHeight="1">
+      <c r="A29" s="112" t="inlineStr">
+        <is>
+          <t>Mobile review-mode seek</t>
+        </is>
+      </c>
+      <c r="B29" s="112" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="C29" s="112" t="inlineStr">
+        <is>
+          <t>The seek bar jump advanced the review timer from 0:07 to 0:28 of 0:37 during playback.</t>
+        </is>
+      </c>
+      <c r="D29" s="112" t="inlineStr">
+        <is>
+          <t>temp/fix-validation-2026-05-07/review-seek-valid.png; temp/fix-validation-2026-05-07/review-seek-valid.xml</t>
+        </is>
+      </c>
+      <c r="E29" s="112" t="inlineStr">
+        <is>
+          <t>This rerun replaced the earlier noisy capture with a clean valid PNG for the appendix.</t>
         </is>
       </c>
     </row>

</xml_diff>